<commit_message>
Day side orbits and minor fixes
</commit_message>
<xml_diff>
--- a/Data Files/MANTIS_Mission_Config_v2.xlsx
+++ b/Data Files/MANTIS_Mission_Config_v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sebastianescobar/Desktop/CubeSatMissionPlanner/Data Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18F93B25-EEFD-CD41-93E5-9675A100DBE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{847DEB99-53CE-6D45-9F20-62D733B0F8C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3840" yWindow="2260" windowWidth="21760" windowHeight="14380" tabRatio="500" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3840" yWindow="2260" windowWidth="21760" windowHeight="14380" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PlanPropagation_Info" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="81">
   <si>
     <t>TLE URL</t>
   </si>
@@ -63,9 +63,6 @@
     <t>Timestep [sec]</t>
   </si>
   <si>
-    <t>https://celestrak.org/NORAD/elements/gp.php?GROUP=active&amp;FORMAT=tle</t>
-  </si>
-  <si>
     <t>cute_tle</t>
   </si>
   <si>
@@ -174,90 +171,12 @@
     <t>EV Lac</t>
   </si>
   <si>
-    <t>Tau Ceti</t>
-  </si>
-  <si>
-    <t>Procyon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HD 189733 </t>
-  </si>
-  <si>
     <t>JUMP</t>
   </si>
   <si>
-    <t xml:space="preserve">55 Cnc </t>
-  </si>
-  <si>
-    <t xml:space="preserve">GJ 357 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">L 98-59 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">WASP-178 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">V1298 Tau </t>
-  </si>
-  <si>
-    <t>HD 209458b</t>
-  </si>
-  <si>
-    <t>LTT 1445A</t>
-  </si>
-  <si>
-    <t>GJ 486</t>
-  </si>
-  <si>
-    <t>GJ 367</t>
-  </si>
-  <si>
-    <t>GJ 341</t>
-  </si>
-  <si>
-    <t>GJ 4102</t>
-  </si>
-  <si>
-    <t>TOI-260</t>
-  </si>
-  <si>
-    <t>TOI-776</t>
-  </si>
-  <si>
-    <t>TOI-836</t>
-  </si>
-  <si>
-    <t>TOI-402</t>
-  </si>
-  <si>
-    <t>HD 80606</t>
-  </si>
-  <si>
-    <t>TOI-421</t>
-  </si>
-  <si>
-    <t>WASP-166</t>
-  </si>
-  <si>
-    <t>WASP-121</t>
-  </si>
-  <si>
-    <t>G191-B2B</t>
-  </si>
-  <si>
     <t>Calibration</t>
   </si>
   <si>
-    <t>GD 71</t>
-  </si>
-  <si>
-    <t>GD 153</t>
-  </si>
-  <si>
-    <t>HZ 43</t>
-  </si>
-  <si>
     <t>N Targets</t>
   </si>
   <si>
@@ -364,6 +283,9 @@
   </si>
   <si>
     <t>A</t>
+  </si>
+  <si>
+    <t>https://celestrak.org/NORAD/elements/gp.php?CATNR=49263&amp;FORMAT=tle</t>
   </si>
 </sst>
 </file>
@@ -375,7 +297,7 @@
     <numFmt numFmtId="165" formatCode="00"/>
     <numFmt numFmtId="166" formatCode="00.000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -413,6 +335,14 @@
       <sz val="14"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -455,10 +385,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -526,8 +457,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -961,14 +895,14 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="31" t="s">
+        <v>80</v>
+      </c>
+      <c r="B2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>7</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>8</v>
       </c>
       <c r="D2" s="5">
         <v>45748.020833333336</v>
@@ -981,6 +915,9 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" tooltip="https://nam10.safelinks.protection.outlook.com/?url=https%3A%2F%2Fcelestrak.org%2FNORAD%2Felements%2Fgp.php%3FCATNR%3D49263%26FORMAT%3Dtle&amp;data=05%7C02%7CSebastian.Escobar%40lasp.colorado.edu%7Cc8b62e77ac294876c08408de9c9ed44c%7Cb1ddd7831dbc446b878fa7b03478ea9e%7C1%7C0%7C639120403139812220%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=u3QfNw08NJ2Lc8RuYxyuN00h4d4s%2FdYbxVHUa8yHL4o%3D&amp;reserved=0" display="https://nam10.safelinks.protection.outlook.com/?url=https%3A%2F%2Fcelestrak.org%2FNORAD%2Felements%2Fgp.php%3FCATNR%3D49263%26FORMAT%3Dtle&amp;data=05%7C02%7CSebastian.Escobar%40lasp.colorado.edu%7Cc8b62e77ac294876c08408de9c9ed44c%7Cb1ddd7831dbc446b878fa7b03478ea9e%7C1%7C0%7C639120403139812220%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=u3QfNw08NJ2Lc8RuYxyuN00h4d4s%2FdYbxVHUa8yHL4o%3D&amp;reserved=0" xr:uid="{1D51D9A4-B8BF-6D47-8F6C-DF94280B8DEE}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -1012,57 +949,57 @@
   <sheetData>
     <row r="1" spans="1:15" s="23" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B1" s="9" t="s">
+      <c r="C1" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="20" t="s">
+      <c r="D1" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="E1" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="F1" s="20" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="G1" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="G1" s="20" t="s">
+      <c r="H1" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="H1" s="21" t="s">
+      <c r="I1" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="M1" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="M1" s="22" t="s">
+      <c r="N1" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>22</v>
-      </c>
-      <c r="O1" s="9" t="s">
-        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C2" s="24">
         <v>10</v>
@@ -1086,7 +1023,7 @@
         <v>0</v>
       </c>
       <c r="J2" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K2" s="12">
         <v>1</v>
@@ -1109,10 +1046,10 @@
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C3" s="24">
         <v>18</v>
@@ -1136,7 +1073,7 @@
         <v>0</v>
       </c>
       <c r="J3" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K3" s="12">
         <v>1</v>
@@ -1159,10 +1096,10 @@
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C4" s="24">
         <v>23</v>
@@ -1186,7 +1123,7 @@
         <v>0</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K4" s="12">
         <v>1</v>
@@ -1209,10 +1146,10 @@
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C5" s="24">
         <v>1</v>
@@ -1236,7 +1173,7 @@
         <v>0</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K5" s="12">
         <v>1</v>
@@ -1259,10 +1196,10 @@
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C6" s="24">
         <v>21</v>
@@ -1286,7 +1223,7 @@
         <v>0</v>
       </c>
       <c r="J6" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K6" s="12">
         <v>1</v>
@@ -1309,10 +1246,10 @@
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C7" s="24">
         <v>6</v>
@@ -1336,7 +1273,7 @@
         <v>0</v>
       </c>
       <c r="J7" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K7" s="12">
         <v>1</v>
@@ -1359,10 +1296,10 @@
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C8" s="24">
         <v>5</v>
@@ -1386,7 +1323,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K8" s="12">
         <v>1</v>
@@ -1409,10 +1346,10 @@
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C9" s="24">
         <v>4</v>
@@ -1436,7 +1373,7 @@
         <v>0</v>
       </c>
       <c r="J9" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K9" s="12">
         <v>1</v>
@@ -1459,10 +1396,10 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C10" s="24">
         <v>10</v>
@@ -1486,7 +1423,7 @@
         <v>0</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K10" s="12">
         <v>1</v>
@@ -1509,10 +1446,10 @@
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C11" s="24">
         <v>3</v>
@@ -1536,7 +1473,7 @@
         <v>0</v>
       </c>
       <c r="J11" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K11" s="12">
         <v>1</v>
@@ -1559,10 +1496,10 @@
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C12" s="24">
         <v>22</v>
@@ -1586,7 +1523,7 @@
         <v>0</v>
       </c>
       <c r="J12" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K12" s="12">
         <v>1</v>
@@ -1609,10 +1546,10 @@
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C13" s="24">
         <v>4</v>
@@ -1636,7 +1573,7 @@
         <v>0</v>
       </c>
       <c r="J13" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K13" s="12">
         <v>1</v>
@@ -1659,10 +1596,10 @@
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C14" s="24">
         <v>8</v>
@@ -1686,7 +1623,7 @@
         <v>0</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K14" s="12">
         <v>1</v>
@@ -1709,10 +1646,10 @@
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A15" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C15" s="24">
         <v>4</v>
@@ -1736,7 +1673,7 @@
         <v>0</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K15" s="12">
         <v>1</v>
@@ -1759,10 +1696,10 @@
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A16" s="14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C16" s="14">
         <v>9</v>
@@ -1786,7 +1723,7 @@
         <v>0</v>
       </c>
       <c r="J16" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K16" s="12">
         <v>1</v>
@@ -1809,10 +1746,10 @@
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A17" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C17" s="14">
         <v>13</v>
@@ -1836,7 +1773,7 @@
         <v>0</v>
       </c>
       <c r="J17" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K17" s="12">
         <v>1</v>
@@ -1859,10 +1796,10 @@
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A18" s="14" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C18" s="14">
         <v>4</v>
@@ -1886,7 +1823,7 @@
         <v>0</v>
       </c>
       <c r="J18" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K18" s="12">
         <v>1</v>
@@ -1909,10 +1846,10 @@
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A19" s="14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>106</v>
+        <v>79</v>
       </c>
       <c r="C19" s="14">
         <v>22</v>
@@ -1936,7 +1873,7 @@
         <v>0</v>
       </c>
       <c r="J19" s="12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K19" s="12">
         <v>1</v>
@@ -1958,1303 +1895,446 @@
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C20" s="14">
-        <v>1</v>
-      </c>
-      <c r="D20" s="14">
-        <v>44</v>
-      </c>
-      <c r="E20" s="14">
-        <v>4.3800940711717802</v>
-      </c>
-      <c r="F20" s="14">
-        <v>-15</v>
-      </c>
-      <c r="G20" s="14">
-        <v>56</v>
-      </c>
-      <c r="H20" s="14">
-        <v>32.357259787263501</v>
-      </c>
-      <c r="I20" s="12">
-        <v>0</v>
-      </c>
-      <c r="J20" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="K20" s="12">
-        <v>1</v>
-      </c>
-      <c r="L20" s="12" t="str">
-        <f>LOOKUP(J20,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M20" s="12">
-        <f>LOOKUP(J20,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N20" s="12">
-        <f>LOOKUP(J20,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O20" s="12">
-        <v>0</v>
-      </c>
+      <c r="A20" s="14"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="12"/>
+      <c r="J20" s="12"/>
+      <c r="K20" s="12"/>
+      <c r="L20" s="12"/>
+      <c r="M20" s="12"/>
+      <c r="N20" s="12"/>
+      <c r="O20" s="12"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C21" s="14">
-        <v>7</v>
-      </c>
-      <c r="D21" s="14">
-        <v>39</v>
-      </c>
-      <c r="E21" s="14">
-        <v>17.7574773317458</v>
-      </c>
-      <c r="F21" s="14">
-        <v>5</v>
-      </c>
-      <c r="G21" s="14">
-        <v>14</v>
-      </c>
-      <c r="H21" s="14">
-        <v>14.713134425050599</v>
-      </c>
-      <c r="I21" s="12">
-        <v>0</v>
-      </c>
-      <c r="J21" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="K21" s="12">
-        <v>1</v>
-      </c>
-      <c r="L21" s="12" t="str">
-        <f>LOOKUP(J21,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M21" s="12">
-        <f>LOOKUP(J21,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N21" s="12">
-        <f>LOOKUP(J21,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O21" s="12">
-        <v>0</v>
-      </c>
+      <c r="A21" s="14"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="14"/>
+      <c r="D21" s="14"/>
+      <c r="E21" s="14"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="14"/>
+      <c r="H21" s="14"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+      <c r="L21" s="12"/>
+      <c r="M21" s="12"/>
+      <c r="N21" s="12"/>
+      <c r="O21" s="12"/>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A22" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C22" s="14">
-        <v>20</v>
-      </c>
-      <c r="D22" s="14">
-        <v>0</v>
-      </c>
-      <c r="E22" s="14">
-        <v>43.712899999999998</v>
-      </c>
-      <c r="F22" s="14">
-        <v>22</v>
-      </c>
-      <c r="G22" s="14">
-        <v>42</v>
-      </c>
-      <c r="H22" s="14">
-        <v>39.073</v>
-      </c>
-      <c r="I22" s="12">
-        <v>0</v>
-      </c>
-      <c r="J22" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K22" s="12">
-        <v>1</v>
-      </c>
-      <c r="L22" s="12" t="str">
-        <f>LOOKUP(J22,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M22" s="12">
-        <f>LOOKUP(J22,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N22" s="12">
-        <f>LOOKUP(J22,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O22" s="12">
-        <v>0</v>
-      </c>
+      <c r="A22" s="14"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="14"/>
+      <c r="D22" s="14"/>
+      <c r="E22" s="14"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="14"/>
+      <c r="H22" s="14"/>
+      <c r="I22" s="12"/>
+      <c r="J22" s="14"/>
+      <c r="K22" s="12"/>
+      <c r="L22" s="12"/>
+      <c r="M22" s="12"/>
+      <c r="N22" s="12"/>
+      <c r="O22" s="12"/>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C23" s="14">
-        <v>8</v>
-      </c>
-      <c r="D23" s="14">
-        <v>52</v>
-      </c>
-      <c r="E23" s="14">
-        <v>35.811100000000003</v>
-      </c>
-      <c r="F23" s="14">
-        <v>28</v>
-      </c>
-      <c r="G23" s="14">
-        <v>19</v>
-      </c>
-      <c r="H23" s="14">
-        <v>50.954000000000001</v>
-      </c>
-      <c r="I23" s="12">
-        <v>0</v>
-      </c>
-      <c r="J23" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K23" s="12">
-        <v>1</v>
-      </c>
-      <c r="L23" s="12" t="str">
-        <f>LOOKUP(J23,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M23" s="12">
-        <f>LOOKUP(J23,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N23" s="12">
-        <f>LOOKUP(J23,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O23" s="12">
-        <v>0</v>
-      </c>
+      <c r="A23" s="14"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="14"/>
+      <c r="E23" s="14"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="14"/>
+      <c r="H23" s="14"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="14"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="12"/>
+      <c r="M23" s="12"/>
+      <c r="N23" s="12"/>
+      <c r="O23" s="12"/>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="14" t="s">
-        <v>48</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C24" s="14">
-        <v>9</v>
-      </c>
-      <c r="D24" s="14">
-        <v>36</v>
-      </c>
-      <c r="E24" s="14">
-        <v>1.6372</v>
-      </c>
-      <c r="F24" s="14">
-        <v>-21</v>
-      </c>
-      <c r="G24" s="14">
-        <v>39</v>
-      </c>
-      <c r="H24" s="14">
-        <v>38.877000000000002</v>
-      </c>
-      <c r="I24" s="12">
-        <v>0</v>
-      </c>
-      <c r="J24" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K24" s="12">
-        <v>1</v>
-      </c>
-      <c r="L24" s="12" t="str">
-        <f>LOOKUP(J24,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M24" s="12">
-        <f>LOOKUP(J24,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N24" s="12">
-        <f>LOOKUP(J24,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O24" s="12">
-        <v>0</v>
-      </c>
+      <c r="A24" s="14"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="14"/>
+      <c r="D24" s="14"/>
+      <c r="E24" s="14"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="14"/>
+      <c r="H24" s="14"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="14"/>
+      <c r="K24" s="12"/>
+      <c r="L24" s="12"/>
+      <c r="M24" s="12"/>
+      <c r="N24" s="12"/>
+      <c r="O24" s="12"/>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C25" s="14">
-        <v>8</v>
-      </c>
-      <c r="D25" s="14">
-        <v>18</v>
-      </c>
-      <c r="E25" s="14">
-        <v>7.6214000000000004</v>
-      </c>
-      <c r="F25" s="14">
-        <v>-68</v>
-      </c>
-      <c r="G25" s="14">
-        <v>18</v>
-      </c>
-      <c r="H25" s="14">
-        <v>46.805</v>
-      </c>
-      <c r="I25" s="12">
-        <v>0</v>
-      </c>
-      <c r="J25" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K25" s="12">
-        <v>1</v>
-      </c>
-      <c r="L25" s="12" t="str">
-        <f>LOOKUP(J25,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M25" s="12">
-        <f>LOOKUP(J25,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N25" s="12">
-        <f>LOOKUP(J25,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O25" s="12">
-        <v>0</v>
-      </c>
+      <c r="A25" s="14"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="14"/>
+      <c r="D25" s="14"/>
+      <c r="E25" s="14"/>
+      <c r="F25" s="14"/>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="14"/>
+      <c r="K25" s="12"/>
+      <c r="L25" s="12"/>
+      <c r="M25" s="12"/>
+      <c r="N25" s="12"/>
+      <c r="O25" s="12"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C26" s="14">
-        <v>15</v>
-      </c>
-      <c r="D26" s="14">
-        <v>9</v>
-      </c>
-      <c r="E26" s="14">
-        <v>4.8933</v>
-      </c>
-      <c r="F26" s="14">
-        <v>-42</v>
-      </c>
-      <c r="G26" s="14">
-        <v>42</v>
-      </c>
-      <c r="H26" s="14">
-        <v>17.789000000000001</v>
-      </c>
-      <c r="I26" s="12">
-        <v>0</v>
-      </c>
-      <c r="J26" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K26" s="12">
-        <v>1</v>
-      </c>
-      <c r="L26" s="12" t="str">
-        <f>LOOKUP(J26,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M26" s="12">
-        <f>LOOKUP(J26,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N26" s="12">
-        <f>LOOKUP(J26,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O26" s="12">
-        <v>0</v>
-      </c>
+      <c r="A26" s="14"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="14"/>
+      <c r="D26" s="14"/>
+      <c r="E26" s="14"/>
+      <c r="F26" s="14"/>
+      <c r="G26" s="14"/>
+      <c r="H26" s="14"/>
+      <c r="I26" s="12"/>
+      <c r="J26" s="14"/>
+      <c r="K26" s="12"/>
+      <c r="L26" s="12"/>
+      <c r="M26" s="12"/>
+      <c r="N26" s="12"/>
+      <c r="O26" s="12"/>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C27" s="14">
-        <v>4</v>
-      </c>
-      <c r="D27" s="14">
-        <v>5</v>
-      </c>
-      <c r="E27" s="14">
-        <v>19.590900000000001</v>
-      </c>
-      <c r="F27" s="14">
-        <v>20</v>
-      </c>
-      <c r="G27" s="14">
-        <v>9</v>
-      </c>
-      <c r="H27" s="14">
-        <v>25.562999999999999</v>
-      </c>
-      <c r="I27" s="12">
-        <v>0</v>
-      </c>
-      <c r="J27" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K27" s="12">
-        <v>1</v>
-      </c>
-      <c r="L27" s="12" t="str">
-        <f>LOOKUP(J27,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M27" s="12">
-        <f>LOOKUP(J27,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N27" s="12">
-        <f>LOOKUP(J27,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O27" s="12">
-        <v>0</v>
-      </c>
+      <c r="A27" s="14"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+      <c r="E27" s="14"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="14"/>
+      <c r="H27" s="14"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="14"/>
+      <c r="K27" s="12"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="12"/>
+      <c r="N27" s="12"/>
+      <c r="O27" s="12"/>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A28" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C28" s="14">
-        <v>22</v>
-      </c>
-      <c r="D28" s="14">
-        <v>3</v>
-      </c>
-      <c r="E28" s="14">
-        <v>10.7727</v>
-      </c>
-      <c r="F28" s="14">
-        <v>18</v>
-      </c>
-      <c r="G28" s="14">
-        <v>53</v>
-      </c>
-      <c r="H28" s="14">
-        <v>3.5489999999999999</v>
-      </c>
-      <c r="I28" s="12">
-        <v>0</v>
-      </c>
-      <c r="J28" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K28" s="12">
-        <v>1</v>
-      </c>
-      <c r="L28" s="12" t="str">
-        <f>LOOKUP(J28,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M28" s="12">
-        <f>LOOKUP(J28,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N28" s="12">
-        <f>LOOKUP(J28,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O28" s="12">
-        <v>0</v>
-      </c>
+      <c r="A28" s="14"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="14"/>
+      <c r="D28" s="14"/>
+      <c r="E28" s="14"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="14"/>
+      <c r="H28" s="14"/>
+      <c r="I28" s="12"/>
+      <c r="J28" s="14"/>
+      <c r="K28" s="12"/>
+      <c r="L28" s="12"/>
+      <c r="M28" s="12"/>
+      <c r="N28" s="12"/>
+      <c r="O28" s="12"/>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A29" s="14" t="s">
-        <v>53</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C29" s="14">
-        <v>3</v>
-      </c>
-      <c r="D29" s="14">
-        <v>1</v>
-      </c>
-      <c r="E29" s="14">
-        <v>51.393599999999999</v>
-      </c>
-      <c r="F29" s="14">
-        <v>-16</v>
-      </c>
-      <c r="G29" s="14">
-        <v>35</v>
-      </c>
-      <c r="H29" s="14">
-        <v>36.030999999999999</v>
-      </c>
-      <c r="I29" s="12">
-        <v>0</v>
-      </c>
-      <c r="J29" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K29" s="12">
-        <v>1</v>
-      </c>
-      <c r="L29" s="12" t="str">
-        <f>LOOKUP(J29,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M29" s="12">
-        <f>LOOKUP(J29,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N29" s="12">
-        <f>LOOKUP(J29,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O29" s="12">
-        <v>0</v>
-      </c>
+      <c r="A29" s="14"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="14"/>
+      <c r="D29" s="14"/>
+      <c r="E29" s="14"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="14"/>
+      <c r="H29" s="14"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="14"/>
+      <c r="K29" s="12"/>
+      <c r="L29" s="12"/>
+      <c r="M29" s="12"/>
+      <c r="N29" s="12"/>
+      <c r="O29" s="12"/>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A30" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C30" s="14">
-        <v>12</v>
-      </c>
-      <c r="D30" s="14">
-        <v>47</v>
-      </c>
-      <c r="E30" s="14">
-        <v>56.624499999999998</v>
-      </c>
-      <c r="F30" s="14">
-        <v>9</v>
-      </c>
-      <c r="G30" s="14">
-        <v>45</v>
-      </c>
-      <c r="H30" s="14">
-        <v>5.0350000000000001</v>
-      </c>
-      <c r="I30" s="12">
-        <v>0</v>
-      </c>
-      <c r="J30" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K30" s="12">
-        <v>1</v>
-      </c>
-      <c r="L30" s="12" t="str">
-        <f>LOOKUP(J30,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M30" s="12">
-        <f>LOOKUP(J30,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N30" s="12">
-        <f>LOOKUP(J30,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O30" s="12">
-        <v>0</v>
-      </c>
+      <c r="A30" s="14"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="14"/>
+      <c r="D30" s="14"/>
+      <c r="E30" s="14"/>
+      <c r="F30" s="14"/>
+      <c r="G30" s="14"/>
+      <c r="H30" s="14"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="14"/>
+      <c r="K30" s="12"/>
+      <c r="L30" s="12"/>
+      <c r="M30" s="12"/>
+      <c r="N30" s="12"/>
+      <c r="O30" s="12"/>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A31" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C31" s="14">
-        <v>9</v>
-      </c>
-      <c r="D31" s="14">
-        <v>44</v>
-      </c>
-      <c r="E31" s="14">
-        <v>29.8367</v>
-      </c>
-      <c r="F31" s="14">
-        <v>-45</v>
-      </c>
-      <c r="G31" s="14">
-        <v>46</v>
-      </c>
-      <c r="H31" s="14">
-        <v>35.427</v>
-      </c>
-      <c r="I31" s="12">
-        <v>0</v>
-      </c>
-      <c r="J31" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K31" s="12">
-        <v>1</v>
-      </c>
-      <c r="L31" s="12" t="str">
-        <f>LOOKUP(J31,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M31" s="12">
-        <f>LOOKUP(J31,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N31" s="12">
-        <f>LOOKUP(J31,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O31" s="12">
-        <v>0</v>
-      </c>
+      <c r="A31" s="14"/>
+      <c r="B31" s="12"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="14"/>
+      <c r="E31" s="14"/>
+      <c r="F31" s="14"/>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="14"/>
+      <c r="K31" s="12"/>
+      <c r="L31" s="12"/>
+      <c r="M31" s="12"/>
+      <c r="N31" s="12"/>
+      <c r="O31" s="12"/>
     </row>
     <row r="32" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A32" s="14" t="s">
-        <v>56</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C32" s="14">
-        <v>9</v>
-      </c>
-      <c r="D32" s="14">
-        <v>21</v>
-      </c>
-      <c r="E32" s="14">
-        <v>37.601500000000001</v>
-      </c>
-      <c r="F32" s="14">
-        <v>-60</v>
-      </c>
-      <c r="G32" s="14">
-        <v>16</v>
-      </c>
-      <c r="H32" s="14">
-        <v>55.03</v>
-      </c>
-      <c r="I32" s="12">
-        <v>0</v>
-      </c>
-      <c r="J32" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K32" s="12">
-        <v>1</v>
-      </c>
-      <c r="L32" s="12" t="str">
-        <f>LOOKUP(J32,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M32" s="12">
-        <f>LOOKUP(J32,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N32" s="12">
-        <f>LOOKUP(J32,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O32" s="12">
-        <v>0</v>
-      </c>
+      <c r="A32" s="14"/>
+      <c r="B32" s="12"/>
+      <c r="C32" s="14"/>
+      <c r="D32" s="14"/>
+      <c r="E32" s="14"/>
+      <c r="F32" s="14"/>
+      <c r="G32" s="14"/>
+      <c r="H32" s="14"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="14"/>
+      <c r="K32" s="12"/>
+      <c r="L32" s="12"/>
+      <c r="M32" s="12"/>
+      <c r="N32" s="12"/>
+      <c r="O32" s="12"/>
     </row>
     <row r="33" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A33" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C33" s="14">
-        <v>19</v>
-      </c>
-      <c r="D33" s="14">
-        <v>20</v>
-      </c>
-      <c r="E33" s="14">
-        <v>54.376100000000001</v>
-      </c>
-      <c r="F33" s="14">
-        <v>-82</v>
-      </c>
-      <c r="G33" s="14">
-        <v>33</v>
-      </c>
-      <c r="H33" s="14">
-        <v>16.167000000000002</v>
-      </c>
-      <c r="I33" s="12">
-        <v>0</v>
-      </c>
-      <c r="J33" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K33" s="12">
-        <v>1</v>
-      </c>
-      <c r="L33" s="12" t="str">
-        <f>LOOKUP(J33,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M33" s="12">
-        <f>LOOKUP(J33,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N33" s="12">
-        <f>LOOKUP(J33,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O33" s="12">
-        <v>0</v>
-      </c>
+      <c r="A33" s="14"/>
+      <c r="B33" s="12"/>
+      <c r="C33" s="14"/>
+      <c r="D33" s="14"/>
+      <c r="E33" s="14"/>
+      <c r="F33" s="14"/>
+      <c r="G33" s="14"/>
+      <c r="H33" s="14"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="14"/>
+      <c r="K33" s="12"/>
+      <c r="L33" s="12"/>
+      <c r="M33" s="12"/>
+      <c r="N33" s="12"/>
+      <c r="O33" s="12"/>
     </row>
     <row r="34" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A34" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C34" s="14">
-        <v>0</v>
-      </c>
-      <c r="D34" s="14">
-        <v>19</v>
-      </c>
-      <c r="E34" s="14">
-        <v>5.5622999999999996</v>
-      </c>
-      <c r="F34" s="14">
-        <v>-9</v>
-      </c>
-      <c r="G34" s="14">
-        <v>57</v>
-      </c>
-      <c r="H34" s="14">
-        <v>53.468000000000004</v>
-      </c>
-      <c r="I34" s="12">
-        <v>0</v>
-      </c>
-      <c r="J34" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K34" s="12">
-        <v>1</v>
-      </c>
-      <c r="L34" s="12" t="str">
-        <f>LOOKUP(J34,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M34" s="12">
-        <f>LOOKUP(J34,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N34" s="12">
-        <f>LOOKUP(J34,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O34" s="12">
-        <v>0</v>
-      </c>
+      <c r="A34" s="14"/>
+      <c r="B34" s="12"/>
+      <c r="C34" s="14"/>
+      <c r="D34" s="14"/>
+      <c r="E34" s="14"/>
+      <c r="F34" s="14"/>
+      <c r="G34" s="14"/>
+      <c r="H34" s="14"/>
+      <c r="I34" s="12"/>
+      <c r="J34" s="14"/>
+      <c r="K34" s="12"/>
+      <c r="L34" s="12"/>
+      <c r="M34" s="12"/>
+      <c r="N34" s="12"/>
+      <c r="O34" s="12"/>
     </row>
     <row r="35" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A35" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C35" s="14">
-        <v>11</v>
-      </c>
-      <c r="D35" s="14">
-        <v>54</v>
-      </c>
-      <c r="E35" s="14">
-        <v>18.392099999999999</v>
-      </c>
-      <c r="F35" s="14">
-        <v>-37</v>
-      </c>
-      <c r="G35" s="14">
-        <v>33</v>
-      </c>
-      <c r="H35" s="14">
-        <v>9.8369999999999997</v>
-      </c>
-      <c r="I35" s="12">
-        <v>0</v>
-      </c>
-      <c r="J35" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K35" s="12">
-        <v>1</v>
-      </c>
-      <c r="L35" s="12" t="str">
-        <f>LOOKUP(J35,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M35" s="12">
-        <f>LOOKUP(J35,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N35" s="12">
-        <f>LOOKUP(J35,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O35" s="12">
-        <v>0</v>
-      </c>
+      <c r="A35" s="14"/>
+      <c r="B35" s="12"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="14"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14"/>
+      <c r="G35" s="14"/>
+      <c r="H35" s="14"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="14"/>
+      <c r="K35" s="12"/>
+      <c r="L35" s="12"/>
+      <c r="M35" s="12"/>
+      <c r="N35" s="12"/>
+      <c r="O35" s="12"/>
     </row>
     <row r="36" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A36" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="B36" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C36" s="14">
-        <v>15</v>
-      </c>
-      <c r="D36" s="14">
-        <v>0</v>
-      </c>
-      <c r="E36" s="14">
-        <v>19.398299999999999</v>
-      </c>
-      <c r="F36" s="14">
-        <v>-24</v>
-      </c>
-      <c r="G36" s="14">
-        <v>27</v>
-      </c>
-      <c r="H36" s="14">
-        <v>14.693</v>
-      </c>
-      <c r="I36" s="12">
-        <v>0</v>
-      </c>
-      <c r="J36" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K36" s="12">
-        <v>-1</v>
-      </c>
-      <c r="L36" s="12" t="str">
-        <f>LOOKUP(J36,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M36" s="12">
-        <v>10000</v>
-      </c>
-      <c r="N36" s="12">
-        <f>LOOKUP(J36,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O36" s="12">
-        <v>0</v>
-      </c>
+      <c r="A36" s="14"/>
+      <c r="B36" s="12"/>
+      <c r="C36" s="14"/>
+      <c r="D36" s="14"/>
+      <c r="E36" s="14"/>
+      <c r="F36" s="14"/>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
+      <c r="I36" s="12"/>
+      <c r="J36" s="14"/>
+      <c r="K36" s="12"/>
+      <c r="L36" s="12"/>
+      <c r="M36" s="12"/>
+      <c r="N36" s="12"/>
+      <c r="O36" s="12"/>
     </row>
     <row r="37" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A37" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C37" s="14">
-        <v>2</v>
-      </c>
-      <c r="D37" s="14">
-        <v>27</v>
-      </c>
-      <c r="E37" s="14">
-        <v>28.3781</v>
-      </c>
-      <c r="F37" s="14">
-        <v>-27</v>
-      </c>
-      <c r="G37" s="14">
-        <v>38</v>
-      </c>
-      <c r="H37" s="14">
-        <v>6.7359999999999998</v>
-      </c>
-      <c r="I37" s="12">
-        <v>0</v>
-      </c>
-      <c r="J37" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K37" s="12">
-        <v>1</v>
-      </c>
-      <c r="L37" s="12" t="str">
-        <f>LOOKUP(J37,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M37" s="12">
-        <f>LOOKUP(J37,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N37" s="12">
-        <f>LOOKUP(J37,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O37" s="12">
-        <v>0</v>
-      </c>
+      <c r="A37" s="14"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="14"/>
+      <c r="D37" s="14"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="14"/>
+      <c r="I37" s="12"/>
+      <c r="J37" s="14"/>
+      <c r="K37" s="12"/>
+      <c r="L37" s="12"/>
+      <c r="M37" s="12"/>
+      <c r="N37" s="12"/>
+      <c r="O37" s="12"/>
     </row>
     <row r="38" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A38" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="B38" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C38" s="14">
-        <v>9</v>
-      </c>
-      <c r="D38" s="14">
-        <v>22</v>
-      </c>
-      <c r="E38" s="14">
-        <v>37.576799999999999</v>
-      </c>
-      <c r="F38" s="14">
-        <v>50</v>
-      </c>
-      <c r="G38" s="14">
-        <v>36</v>
-      </c>
-      <c r="H38" s="14">
-        <v>13.435</v>
-      </c>
-      <c r="I38" s="12">
-        <v>0</v>
-      </c>
-      <c r="J38" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K38" s="12">
-        <v>1</v>
-      </c>
-      <c r="L38" s="12" t="str">
-        <f>LOOKUP(J38,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M38" s="12">
-        <f>LOOKUP(J38,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N38" s="12">
-        <f>LOOKUP(J38,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O38" s="12">
-        <v>0</v>
-      </c>
+      <c r="A38" s="14"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="14"/>
+      <c r="D38" s="14"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14"/>
+      <c r="I38" s="12"/>
+      <c r="J38" s="14"/>
+      <c r="K38" s="12"/>
+      <c r="L38" s="12"/>
+      <c r="M38" s="12"/>
+      <c r="N38" s="12"/>
+      <c r="O38" s="12"/>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A39" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C39" s="14">
-        <v>5</v>
-      </c>
-      <c r="D39" s="14">
-        <v>27</v>
-      </c>
-      <c r="E39" s="14">
-        <v>24.825800000000001</v>
-      </c>
-      <c r="F39" s="14">
-        <v>-14</v>
-      </c>
-      <c r="G39" s="14">
-        <v>16</v>
-      </c>
-      <c r="H39" s="14">
-        <v>37.045999999999999</v>
-      </c>
-      <c r="I39" s="12">
-        <v>0</v>
-      </c>
-      <c r="J39" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K39" s="12">
-        <v>1</v>
-      </c>
-      <c r="L39" s="12" t="str">
-        <f>LOOKUP(J39,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M39" s="12">
-        <f>LOOKUP(J39,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N39" s="12">
-        <f>LOOKUP(J39,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O39" s="12">
-        <v>0</v>
-      </c>
+      <c r="A39" s="14"/>
+      <c r="B39" s="12"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="14"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="14"/>
+      <c r="H39" s="14"/>
+      <c r="I39" s="12"/>
+      <c r="J39" s="14"/>
+      <c r="K39" s="12"/>
+      <c r="L39" s="12"/>
+      <c r="M39" s="12"/>
+      <c r="N39" s="12"/>
+      <c r="O39" s="12"/>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A40" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C40" s="14">
-        <v>9</v>
-      </c>
-      <c r="D40" s="14">
-        <v>39</v>
-      </c>
-      <c r="E40" s="14">
-        <v>30.086099999999998</v>
-      </c>
-      <c r="F40" s="14">
-        <v>-20</v>
-      </c>
-      <c r="G40" s="14">
-        <v>58</v>
-      </c>
-      <c r="H40" s="14">
-        <v>56.881</v>
-      </c>
-      <c r="I40" s="12">
-        <v>0</v>
-      </c>
-      <c r="J40" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K40" s="12">
-        <v>1</v>
-      </c>
-      <c r="L40" s="12" t="str">
-        <f>LOOKUP(J40,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M40" s="12">
-        <f>LOOKUP(J40,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N40" s="12">
-        <f>LOOKUP(J40,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O40" s="12">
-        <v>0</v>
-      </c>
+      <c r="A40" s="14"/>
+      <c r="B40" s="12"/>
+      <c r="C40" s="14"/>
+      <c r="D40" s="14"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="14"/>
+      <c r="G40" s="14"/>
+      <c r="H40" s="14"/>
+      <c r="I40" s="12"/>
+      <c r="J40" s="14"/>
+      <c r="K40" s="12"/>
+      <c r="L40" s="12"/>
+      <c r="M40" s="12"/>
+      <c r="N40" s="12"/>
+      <c r="O40" s="12"/>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A41" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="B41" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C41" s="14">
-        <v>7</v>
-      </c>
-      <c r="D41" s="14">
-        <v>10</v>
-      </c>
-      <c r="E41" s="14">
-        <v>24.060400000000001</v>
-      </c>
-      <c r="F41" s="14">
-        <v>-39</v>
-      </c>
-      <c r="G41" s="14">
-        <v>5</v>
-      </c>
-      <c r="H41" s="14">
-        <v>50.570999999999998</v>
-      </c>
-      <c r="I41" s="12">
-        <v>0</v>
-      </c>
-      <c r="J41" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="K41" s="12">
-        <v>1</v>
-      </c>
-      <c r="L41" s="12" t="str">
-        <f>LOOKUP(J41,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M41" s="12">
-        <f>LOOKUP(J41,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N41" s="12">
-        <f>LOOKUP(J41,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O41" s="12">
-        <v>0</v>
-      </c>
+      <c r="A41" s="14"/>
+      <c r="B41" s="12"/>
+      <c r="C41" s="14"/>
+      <c r="D41" s="14"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="14"/>
+      <c r="G41" s="14"/>
+      <c r="H41" s="14"/>
+      <c r="I41" s="12"/>
+      <c r="J41" s="14"/>
+      <c r="K41" s="12"/>
+      <c r="L41" s="12"/>
+      <c r="M41" s="12"/>
+      <c r="N41" s="12"/>
+      <c r="O41" s="12"/>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A42" s="14" t="s">
-        <v>66</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C42" s="14">
-        <v>5</v>
-      </c>
-      <c r="D42" s="14">
-        <v>5</v>
-      </c>
-      <c r="E42" s="14">
-        <v>30.6</v>
-      </c>
-      <c r="F42" s="14">
-        <v>52</v>
-      </c>
-      <c r="G42" s="14">
-        <v>49</v>
-      </c>
-      <c r="H42" s="14">
-        <v>54</v>
-      </c>
-      <c r="I42" s="12">
-        <v>0</v>
-      </c>
-      <c r="J42" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="K42" s="12">
-        <v>1</v>
-      </c>
-      <c r="L42" s="12" t="str">
-        <f>LOOKUP(J42,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M42" s="12">
-        <f>LOOKUP(J42,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N42" s="12">
-        <f>LOOKUP(J42,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O42" s="12">
-        <v>0</v>
-      </c>
+      <c r="A42" s="14"/>
+      <c r="B42" s="12"/>
+      <c r="C42" s="14"/>
+      <c r="D42" s="14"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="14"/>
+      <c r="G42" s="14"/>
+      <c r="H42" s="14"/>
+      <c r="I42" s="12"/>
+      <c r="J42" s="14"/>
+      <c r="K42" s="12"/>
+      <c r="L42" s="12"/>
+      <c r="M42" s="12"/>
+      <c r="N42" s="12"/>
+      <c r="O42" s="12"/>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A43" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C43" s="14">
-        <v>5</v>
-      </c>
-      <c r="D43" s="14">
-        <v>52</v>
-      </c>
-      <c r="E43" s="14">
-        <v>27.5</v>
-      </c>
-      <c r="F43" s="14">
-        <v>15</v>
-      </c>
-      <c r="G43" s="14">
-        <v>53</v>
-      </c>
-      <c r="H43" s="14">
-        <v>17</v>
-      </c>
-      <c r="I43" s="12">
-        <v>0</v>
-      </c>
-      <c r="J43" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="K43" s="12">
-        <v>1</v>
-      </c>
-      <c r="L43" s="12" t="str">
-        <f>LOOKUP(J43,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M43" s="12">
-        <f>LOOKUP(J43,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N43" s="12">
-        <f>LOOKUP(J43,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O43" s="12">
-        <v>0</v>
-      </c>
+      <c r="A43" s="14"/>
+      <c r="B43" s="12"/>
+      <c r="C43" s="14"/>
+      <c r="D43" s="14"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="14"/>
+      <c r="G43" s="14"/>
+      <c r="H43" s="14"/>
+      <c r="I43" s="12"/>
+      <c r="J43" s="14"/>
+      <c r="K43" s="12"/>
+      <c r="L43" s="12"/>
+      <c r="M43" s="12"/>
+      <c r="N43" s="12"/>
+      <c r="O43" s="12"/>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A44" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="B44" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C44" s="14">
-        <v>12</v>
-      </c>
-      <c r="D44" s="14">
-        <v>57</v>
-      </c>
-      <c r="E44" s="14">
-        <v>2.4</v>
-      </c>
-      <c r="F44" s="14">
-        <v>22</v>
-      </c>
-      <c r="G44" s="14">
-        <v>1</v>
-      </c>
-      <c r="H44" s="14">
-        <v>56</v>
-      </c>
-      <c r="I44" s="12">
-        <v>0</v>
-      </c>
-      <c r="J44" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="K44" s="12">
-        <v>1</v>
-      </c>
-      <c r="L44" s="12" t="str">
-        <f>LOOKUP(J44,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M44" s="12">
-        <f>LOOKUP(J44,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N44" s="12">
-        <f>LOOKUP(J44,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O44" s="12">
-        <v>0</v>
-      </c>
+      <c r="A44" s="14"/>
+      <c r="B44" s="12"/>
+      <c r="C44" s="14"/>
+      <c r="D44" s="14"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="14"/>
+      <c r="G44" s="14"/>
+      <c r="H44" s="14"/>
+      <c r="I44" s="12"/>
+      <c r="J44" s="14"/>
+      <c r="K44" s="12"/>
+      <c r="L44" s="12"/>
+      <c r="M44" s="12"/>
+      <c r="N44" s="12"/>
+      <c r="O44" s="12"/>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A45" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="B45" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="C45" s="14">
-        <v>13</v>
-      </c>
-      <c r="D45" s="14">
-        <v>16</v>
-      </c>
-      <c r="E45" s="14">
-        <v>22</v>
-      </c>
-      <c r="F45" s="14">
-        <v>29</v>
-      </c>
-      <c r="G45" s="14">
-        <v>5</v>
-      </c>
-      <c r="H45" s="14">
-        <v>57</v>
-      </c>
-      <c r="I45" s="12">
-        <v>0</v>
-      </c>
-      <c r="J45" s="14" t="s">
-        <v>67</v>
-      </c>
-      <c r="K45" s="12">
-        <v>1</v>
-      </c>
-      <c r="L45" s="12" t="str">
-        <f>LOOKUP(J45,Survey_Info!A:A,Survey_Info!G:G)</f>
-        <v>TTAG</v>
-      </c>
-      <c r="M45" s="12">
-        <f>LOOKUP(J45,Survey_Info!A:A,Survey_Info!D:D)</f>
-        <v>10000</v>
-      </c>
-      <c r="N45" s="12">
-        <f>LOOKUP(J45,Survey_Info!A:A, Survey_Info!J:J)</f>
-        <v>1000</v>
-      </c>
-      <c r="O45" s="12">
-        <v>0</v>
-      </c>
+      <c r="A45" s="14"/>
+      <c r="B45" s="12"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="14"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="14"/>
+      <c r="G45" s="14"/>
+      <c r="H45" s="14"/>
+      <c r="I45" s="12"/>
+      <c r="J45" s="14"/>
+      <c r="K45" s="12"/>
+      <c r="L45" s="12"/>
+      <c r="M45" s="12"/>
+      <c r="N45" s="12"/>
+      <c r="O45" s="12"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A46" s="14"/>
@@ -4175,39 +3255,39 @@
   <sheetData>
     <row r="1" spans="1:10" s="11" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>72</v>
+        <v>45</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>73</v>
+        <v>46</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>74</v>
+        <v>47</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>75</v>
+        <v>48</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>76</v>
+        <v>49</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>77</v>
+        <v>50</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>78</v>
+        <v>51</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>79</v>
+        <v>52</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B2" s="13">
         <v>20</v>
@@ -4227,10 +3307,10 @@
         <v>8000000</v>
       </c>
       <c r="G2" s="13" t="s">
-        <v>80</v>
+        <v>53</v>
       </c>
       <c r="H2" s="13" t="s">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="I2" s="13">
         <v>2</v>
@@ -4241,7 +3321,7 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B3" s="13">
         <v>15</v>
@@ -4260,10 +3340,10 @@
         <v>5000000</v>
       </c>
       <c r="G3" s="13" t="s">
-        <v>80</v>
+        <v>53</v>
       </c>
       <c r="H3" s="13" t="s">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="I3" s="13">
         <v>1</v>
@@ -4274,7 +3354,7 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>67</v>
+        <v>43</v>
       </c>
       <c r="B4" s="13">
         <v>4</v>
@@ -4294,10 +3374,10 @@
         <v>80000</v>
       </c>
       <c r="G4" s="13" t="s">
-        <v>80</v>
+        <v>53</v>
       </c>
       <c r="H4" s="13" t="s">
-        <v>105</v>
+        <v>78</v>
       </c>
       <c r="I4" s="13">
         <v>3</v>
@@ -4344,25 +3424,25 @@
   <sheetData>
     <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>81</v>
+        <v>54</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>82</v>
+        <v>55</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>83</v>
+        <v>56</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>84</v>
+        <v>57</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>86</v>
+        <v>59</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>87</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -4414,21 +3494,21 @@
   <sheetData>
     <row r="1" spans="1:7" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>88</v>
+        <v>61</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>89</v>
+        <v>62</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>90</v>
+        <v>63</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>91</v>
+        <v>64</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="F1" s="18"/>
+        <v>65</v>
+      </c>
+      <c r="F1" s="32"/>
       <c r="G1" s="18"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -4436,7 +3516,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="17">
-        <v>200</v>
+        <v>2000</v>
       </c>
       <c r="C2" s="17">
         <v>2</v>
@@ -4464,25 +3544,25 @@
   <sheetData>
     <row r="1" spans="1:6" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>93</v>
+        <v>66</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>95</v>
+        <v>68</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>96</v>
+        <v>69</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="F1" s="18"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
-        <v>98</v>
+        <v>71</v>
       </c>
       <c r="B2" s="17">
         <v>40.015000000000001</v>
@@ -4500,7 +3580,7 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
-        <v>99</v>
+        <v>72</v>
       </c>
       <c r="B3" s="17">
         <v>40.10078</v>
@@ -4517,7 +3597,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="17" t="s">
-        <v>100</v>
+        <v>73</v>
       </c>
       <c r="B4" s="17">
         <v>45.854579999999999</v>
@@ -4534,7 +3614,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="17" t="s">
-        <v>101</v>
+        <v>74</v>
       </c>
       <c r="B5" s="17">
         <v>53.778799999999997</v>
@@ -4562,10 +3642,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="B1" t="s">
-        <v>95</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
@@ -5386,13 +4466,13 @@
   <sheetData>
     <row r="1" spans="1:3" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>102</v>
+        <v>75</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>103</v>
+        <v>76</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>104</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="19" x14ac:dyDescent="0.25">

</xml_diff>